<commit_message>
FIX: HILAB original columns names
</commit_message>
<xml_diff>
--- a/data/rename_columns.xlsx
+++ b/data/rename_columns.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="87">
   <si>
     <t>lab_id</t>
   </si>
@@ -238,10 +238,16 @@
     <t>HILAB</t>
   </si>
   <si>
+    <t>Código Da Cápsula</t>
+  </si>
+  <si>
     <t>Código da Capsula</t>
   </si>
   <si>
     <t>Estado</t>
+  </si>
+  <si>
+    <t>Data Do Exame</t>
   </si>
   <si>
     <t>Data do Exame</t>
@@ -644,7 +650,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="21.005" customWidth="1" bestFit="1"/>
@@ -653,7 +659,7 @@
     <col min="4" max="4" style="4" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -667,7 +673,7 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25" hidden="1">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -679,7 +685,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25" hidden="1">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -691,7 +697,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25" hidden="1">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -703,7 +709,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25" hidden="1">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -715,7 +721,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25" hidden="1">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -727,7 +733,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25" hidden="1">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -739,7 +745,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25" hidden="1">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
@@ -753,7 +759,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25" hidden="1">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
@@ -767,7 +773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25" hidden="1">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
@@ -781,7 +787,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25" hidden="1">
       <c r="A11" s="2" t="s">
         <v>4</v>
       </c>
@@ -795,7 +801,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25" hidden="1">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
@@ -809,7 +815,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25" hidden="1">
       <c r="A13" s="2" t="s">
         <v>4</v>
       </c>
@@ -823,7 +829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25" hidden="1">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
@@ -837,7 +843,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25" hidden="1">
       <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
@@ -851,7 +857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25" hidden="1">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
@@ -865,7 +871,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25" hidden="1">
       <c r="A17" s="2" t="s">
         <v>4</v>
       </c>
@@ -879,7 +885,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25" hidden="1">
       <c r="A18" s="2" t="s">
         <v>4</v>
       </c>
@@ -891,7 +897,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25" hidden="1">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
@@ -903,7 +909,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25" hidden="1">
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
@@ -915,7 +921,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25" hidden="1">
       <c r="A21" s="2" t="s">
         <v>31</v>
       </c>
@@ -927,7 +933,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25" hidden="1">
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
@@ -939,7 +945,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25" hidden="1">
       <c r="A23" s="2" t="s">
         <v>31</v>
       </c>
@@ -951,7 +957,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25" hidden="1">
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
@@ -963,7 +969,7 @@
       </c>
       <c r="D24" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25" hidden="1">
       <c r="A25" s="2" t="s">
         <v>31</v>
       </c>
@@ -975,7 +981,7 @@
       </c>
       <c r="D25" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25" hidden="1">
       <c r="A26" s="2" t="s">
         <v>31</v>
       </c>
@@ -987,7 +993,7 @@
       </c>
       <c r="D26" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25" hidden="1">
       <c r="A27" s="2" t="s">
         <v>31</v>
       </c>
@@ -999,7 +1005,7 @@
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25" hidden="1">
       <c r="A28" s="2" t="s">
         <v>31</v>
       </c>
@@ -1011,7 +1017,7 @@
       </c>
       <c r="D28" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25" hidden="1">
       <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
@@ -1023,7 +1029,7 @@
       </c>
       <c r="D29" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25" hidden="1">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1035,7 +1041,7 @@
       </c>
       <c r="D30" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25" hidden="1">
       <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
@@ -1047,7 +1053,7 @@
       </c>
       <c r="D31" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25" hidden="1">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
@@ -1059,7 +1065,7 @@
       </c>
       <c r="D32" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25" hidden="1">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -1073,7 +1079,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25" hidden="1">
       <c r="A34" s="2" t="s">
         <v>31</v>
       </c>
@@ -1087,7 +1093,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25" hidden="1">
       <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
@@ -1099,7 +1105,7 @@
       </c>
       <c r="D35" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25" hidden="1">
       <c r="A36" s="2" t="s">
         <v>31</v>
       </c>
@@ -1111,7 +1117,7 @@
       </c>
       <c r="D36" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="17.25" hidden="1">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -1123,7 +1129,7 @@
       </c>
       <c r="D37" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="17.25" hidden="1">
       <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
@@ -1135,7 +1141,7 @@
       </c>
       <c r="D38" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="17.25" hidden="1">
       <c r="A39" s="2" t="s">
         <v>31</v>
       </c>
@@ -1147,7 +1153,7 @@
       </c>
       <c r="D39" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="17.25" hidden="1">
       <c r="A40" s="2" t="s">
         <v>31</v>
       </c>
@@ -1159,7 +1165,7 @@
       </c>
       <c r="D40" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="17.25" hidden="1">
       <c r="A41" s="2" t="s">
         <v>31</v>
       </c>
@@ -1173,7 +1179,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="17.25" hidden="1">
       <c r="A42" s="2" t="s">
         <v>31</v>
       </c>
@@ -1187,7 +1193,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="17.25" hidden="1">
       <c r="A43" s="2" t="s">
         <v>31</v>
       </c>
@@ -1201,7 +1207,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="17.25" hidden="1">
       <c r="A44" s="2" t="s">
         <v>31</v>
       </c>
@@ -1215,7 +1221,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="17.25" hidden="1">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
@@ -1229,7 +1235,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="17.25" hidden="1">
       <c r="A46" s="2" t="s">
         <v>31</v>
       </c>
@@ -1243,7 +1249,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="17.25" hidden="1">
       <c r="A47" s="2" t="s">
         <v>31</v>
       </c>
@@ -1257,7 +1263,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="17.25" hidden="1">
       <c r="A48" s="2" t="s">
         <v>63</v>
       </c>
@@ -1269,7 +1275,7 @@
       </c>
       <c r="D48" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="17.25" hidden="1">
       <c r="A49" s="2" t="s">
         <v>63</v>
       </c>
@@ -1281,7 +1287,7 @@
       </c>
       <c r="D49" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="17.25" hidden="1">
       <c r="A50" s="2" t="s">
         <v>63</v>
       </c>
@@ -1293,7 +1299,7 @@
       </c>
       <c r="D50" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="17.25" hidden="1">
       <c r="A51" s="2" t="s">
         <v>63</v>
       </c>
@@ -1305,7 +1311,7 @@
       </c>
       <c r="D51" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="17.25" hidden="1">
       <c r="A52" s="2" t="s">
         <v>63</v>
       </c>
@@ -1317,7 +1323,7 @@
       </c>
       <c r="D52" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="17.25" hidden="1">
       <c r="A53" s="2" t="s">
         <v>63</v>
       </c>
@@ -1329,7 +1335,7 @@
       </c>
       <c r="D53" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="17.25" hidden="1">
       <c r="A54" s="2" t="s">
         <v>63</v>
       </c>
@@ -1361,7 +1367,7 @@
         <v>74</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D56" s="2"/>
     </row>
@@ -1370,10 +1376,10 @@
         <v>72</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D57" s="2"/>
     </row>
@@ -1382,10 +1388,10 @@
         <v>72</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D58" s="2"/>
     </row>
@@ -1394,10 +1400,10 @@
         <v>72</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D59" s="2"/>
     </row>
@@ -1406,10 +1412,10 @@
         <v>72</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D60" s="2"/>
     </row>
@@ -1418,192 +1424,216 @@
         <v>72</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D61" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="17.25">
       <c r="A62" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>78</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="D62" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="17.25">
       <c r="A63" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D63" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="17.25" hidden="1">
+      <c r="A64" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D64" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="17.25" hidden="1">
+      <c r="A65" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="C65" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D63" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="17.25">
-      <c r="A64" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B64" s="2" t="s">
+      <c r="D65" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="17.25" hidden="1">
+      <c r="A66" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="B66" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D64" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="17.25">
-      <c r="A65" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C65" s="2" t="s">
+      <c r="D66" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="17.25" hidden="1">
+      <c r="A67" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D65" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="17.25">
-      <c r="A66" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B66" s="2" t="s">
+      <c r="D67" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="17.25" hidden="1">
+      <c r="A68" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C68" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D66" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="17.25">
-      <c r="A67" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B67" s="2" t="s">
+      <c r="D68" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="17.25" hidden="1">
+      <c r="A69" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C69" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D67" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="17.25">
-      <c r="A68" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D68" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="19.5">
-      <c r="A69" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="D69" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="17.25" hidden="1">
       <c r="A70" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D70" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="17.25" hidden="1">
       <c r="A71" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D71" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="17.25" hidden="1">
+      <c r="A72" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D72" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="17.25" hidden="1">
+      <c r="A73" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D71" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="17.25">
-      <c r="A72" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B72" s="2" t="s">
+      <c r="D73" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="17.25" hidden="1">
+      <c r="A74" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C74" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D72" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="17.25">
-      <c r="A73" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C73" s="2" t="s">
+      <c r="D74" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="17.25" hidden="1">
+      <c r="A75" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D73" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="17.25">
-      <c r="A74" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B74" s="2" t="s">
+      <c r="D75" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="17.25" hidden="1">
+      <c r="A76" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C76" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D74" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="17.25">
-      <c r="A75" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B75" s="2" t="s">
+      <c r="D76" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="17.25" hidden="1">
+      <c r="A77" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="B77" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C77" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D75" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="17.25">
-      <c r="A76" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C76" s="2" t="s">
+      <c r="D77" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="17.25" hidden="1">
+      <c r="A78" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C78" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D76" s="2"/>
+      <c r="D78" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Correction "Goias" HIAE data
</commit_message>
<xml_diff>
--- a/data/rename_columns.xlsx
+++ b/data/rename_columns.xlsx
@@ -1,19 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bragatte/Documents/GitHub/respat/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2E73E7-F72A-7A4D-AB44-60906DBC59EB}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-38400" yWindow="-1460" windowWidth="38400" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Sheet1!$A$1:$D$1</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -25,278 +30,275 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="88">
   <si>
-    <t xml:space="preserve">lab_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">column_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DASA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_exame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date_testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">idade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sexo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">codigorequisicao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">codigo_externo_do_paciente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DASA_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">requisicao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uf_norm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cidade_norm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resultado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SC2_test_result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gene N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_geneN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gene S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_geneS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gene ORF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_ORF1ab</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DB Mol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NumeroPedido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DataNascimento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">birthdate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sexo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DataHoraLiberacaoClinica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLUARV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_FluA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NGRV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSVRV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_VSR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SGRV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLUBRV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_FluB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDRPGRV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_RDRP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EGENERV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_geneE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ct_SARS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NGENE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DB Molecular_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SGENE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORF1AB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZZE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZZN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZZRD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZZS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZZZORF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resultado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLEURY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MUNICIPIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IDADE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESTADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEXO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATA COLETA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODIGO REQUISICAO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PACIENTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">patient_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HILAB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código Da Cápsula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código da Capsula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data Do Exame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data do Exame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HLAGyn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dt. Nascimento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pedido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data Coleta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SABIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DataAtendimento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Municipio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paciente</t>
+    <t>lab_id</t>
+  </si>
+  <si>
+    <t>column_name</t>
+  </si>
+  <si>
+    <t>new_name</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>DASA</t>
+  </si>
+  <si>
+    <t>data_exame</t>
+  </si>
+  <si>
+    <t>date_testing</t>
+  </si>
+  <si>
+    <t>idade</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>sexo</t>
+  </si>
+  <si>
+    <t>sex</t>
+  </si>
+  <si>
+    <t>uf</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>codigorequisicao</t>
+  </si>
+  <si>
+    <t>test_id</t>
+  </si>
+  <si>
+    <t>cidade</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>codigo_externo_do_paciente</t>
+  </si>
+  <si>
+    <t>DASA_2</t>
+  </si>
+  <si>
+    <t>requisicao</t>
+  </si>
+  <si>
+    <t>uf_norm</t>
+  </si>
+  <si>
+    <t>cidade_norm</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>resultado</t>
+  </si>
+  <si>
+    <t>SC2_test_result</t>
+  </si>
+  <si>
+    <t>Gene N</t>
+  </si>
+  <si>
+    <t>Ct_geneN</t>
+  </si>
+  <si>
+    <t>Gene S</t>
+  </si>
+  <si>
+    <t>Ct_geneS</t>
+  </si>
+  <si>
+    <t>Gene ORF</t>
+  </si>
+  <si>
+    <t>Ct_ORF1ab</t>
+  </si>
+  <si>
+    <t>DB Mol</t>
+  </si>
+  <si>
+    <t>NumeroPedido</t>
+  </si>
+  <si>
+    <t>DataNascimento</t>
+  </si>
+  <si>
+    <t>birthdate</t>
+  </si>
+  <si>
+    <t>Sexo</t>
+  </si>
+  <si>
+    <t>Cidade</t>
+  </si>
+  <si>
+    <t>UF</t>
+  </si>
+  <si>
+    <t>DataHoraLiberacaoClinica</t>
+  </si>
+  <si>
+    <t>FLUARV</t>
+  </si>
+  <si>
+    <t>Ct_FluA</t>
+  </si>
+  <si>
+    <t>NGRV</t>
+  </si>
+  <si>
+    <t>RSVRV</t>
+  </si>
+  <si>
+    <t>Ct_VSR</t>
+  </si>
+  <si>
+    <t>SGRV</t>
+  </si>
+  <si>
+    <t>FLUBRV</t>
+  </si>
+  <si>
+    <t>Ct_FluB</t>
+  </si>
+  <si>
+    <t>RDRPGRV</t>
+  </si>
+  <si>
+    <t>Ct_RDRP</t>
+  </si>
+  <si>
+    <t>EGENERV</t>
+  </si>
+  <si>
+    <t>Ct_geneE</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>Ct_SARS</t>
+  </si>
+  <si>
+    <t>NGENE</t>
+  </si>
+  <si>
+    <t>DB Molecular_2</t>
+  </si>
+  <si>
+    <t>SGENE</t>
+  </si>
+  <si>
+    <t>ORF1AB</t>
+  </si>
+  <si>
+    <t>ZZZE</t>
+  </si>
+  <si>
+    <t>ZZZN</t>
+  </si>
+  <si>
+    <t>ZZZRD</t>
+  </si>
+  <si>
+    <t>ZZZS</t>
+  </si>
+  <si>
+    <t>ZZZORF</t>
+  </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>FLEURY</t>
+  </si>
+  <si>
+    <t>MUNICIPIO</t>
+  </si>
+  <si>
+    <t>IDADE</t>
+  </si>
+  <si>
+    <t>ESTADO</t>
+  </si>
+  <si>
+    <t>SEXO</t>
+  </si>
+  <si>
+    <t>DATA COLETA</t>
+  </si>
+  <si>
+    <t>CODIGO REQUISICAO</t>
+  </si>
+  <si>
+    <t>PACIENTE</t>
+  </si>
+  <si>
+    <t>patient_id</t>
+  </si>
+  <si>
+    <t>HILAB</t>
+  </si>
+  <si>
+    <t>Código Da Cápsula</t>
+  </si>
+  <si>
+    <t>Código da Capsula</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Data Do Exame</t>
+  </si>
+  <si>
+    <t>Data do Exame</t>
+  </si>
+  <si>
+    <t>Idade</t>
+  </si>
+  <si>
+    <t>HLAGyn</t>
+  </si>
+  <si>
+    <t>Dt. Nascimento</t>
+  </si>
+  <si>
+    <t>Pedido</t>
+  </si>
+  <si>
+    <t>Data Coleta</t>
+  </si>
+  <si>
+    <t>SABIN</t>
+  </si>
+  <si>
+    <t>DataAtendimento</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>Municipio</t>
+  </si>
+  <si>
+    <t>Paciente</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -305,22 +307,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -350,7 +337,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -358,96 +345,343 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D79"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.14"/>
+    <col min="1" max="1" width="21" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -461,7 +695,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -472,7 +706,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -483,7 +717,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -494,7 +728,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -505,7 +739,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -516,7 +750,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -527,7 +761,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -541,7 +775,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -555,7 +789,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -569,7 +803,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -583,7 +817,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
@@ -597,7 +831,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
@@ -611,7 +845,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
@@ -625,7 +859,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
@@ -639,7 +873,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -653,7 +887,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
@@ -667,7 +901,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -678,7 +912,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -689,7 +923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
@@ -700,7 +934,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
@@ -711,7 +945,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -722,7 +956,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -733,7 +967,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>31</v>
       </c>
@@ -744,7 +978,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -755,7 +989,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>31</v>
       </c>
@@ -766,7 +1000,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>31</v>
       </c>
@@ -777,7 +1011,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>31</v>
       </c>
@@ -788,7 +1022,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
@@ -799,7 +1033,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
@@ -810,7 +1044,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
@@ -821,7 +1055,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
@@ -832,7 +1066,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -846,7 +1080,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>31</v>
       </c>
@@ -860,7 +1094,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>31</v>
       </c>
@@ -871,7 +1105,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>31</v>
       </c>
@@ -882,7 +1116,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>31</v>
       </c>
@@ -893,7 +1127,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>31</v>
       </c>
@@ -904,7 +1138,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>31</v>
       </c>
@@ -915,7 +1149,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>31</v>
       </c>
@@ -926,7 +1160,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>31</v>
       </c>
@@ -940,7 +1174,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>31</v>
       </c>
@@ -954,7 +1188,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>31</v>
       </c>
@@ -968,7 +1202,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>31</v>
       </c>
@@ -982,7 +1216,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>31</v>
       </c>
@@ -996,7 +1230,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>31</v>
       </c>
@@ -1010,7 +1244,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>31</v>
       </c>
@@ -1024,7 +1258,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>63</v>
       </c>
@@ -1035,7 +1269,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>63</v>
       </c>
@@ -1046,7 +1280,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>63</v>
       </c>
@@ -1057,7 +1291,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>63</v>
       </c>
@@ -1068,7 +1302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>63</v>
       </c>
@@ -1079,7 +1313,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>63</v>
       </c>
@@ -1090,7 +1324,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>63</v>
       </c>
@@ -1101,7 +1335,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>72</v>
       </c>
@@ -1112,7 +1346,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>72</v>
       </c>
@@ -1123,7 +1357,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>72</v>
       </c>
@@ -1134,7 +1368,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>72</v>
       </c>
@@ -1145,7 +1379,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>72</v>
       </c>
@@ -1156,7 +1390,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>72</v>
       </c>
@@ -1167,7 +1401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>72</v>
       </c>
@@ -1178,7 +1412,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>72</v>
       </c>
@@ -1189,7 +1423,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>72</v>
       </c>
@@ -1200,7 +1434,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>79</v>
       </c>
@@ -1211,7 +1445,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>79</v>
       </c>
@@ -1222,7 +1456,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>79</v>
       </c>
@@ -1233,7 +1467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>79</v>
       </c>
@@ -1244,7 +1478,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>79</v>
       </c>
@@ -1255,7 +1489,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>79</v>
       </c>
@@ -1266,7 +1500,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>79</v>
       </c>
@@ -1277,7 +1511,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>79</v>
       </c>
@@ -1288,7 +1522,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>83</v>
       </c>
@@ -1299,7 +1533,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>83</v>
       </c>
@@ -1310,7 +1544,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>83</v>
       </c>
@@ -1321,7 +1555,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="75" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>83</v>
       </c>
@@ -1332,7 +1566,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>83</v>
       </c>
@@ -1343,7 +1577,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>83</v>
       </c>
@@ -1354,7 +1588,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="17.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>83</v>
       </c>
@@ -1365,7 +1599,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>72</v>
       </c>
@@ -1377,12 +1611,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
FIX: Use both old and new versions of Dasa raw data
</commit_message>
<xml_diff>
--- a/data/rename_columns.xlsx
+++ b/data/rename_columns.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="95">
   <si>
     <t>lab_id</t>
   </si>
@@ -86,6 +86,21 @@
   </si>
   <si>
     <t>cidade</t>
+  </si>
+  <si>
+    <t>Patógeno</t>
+  </si>
+  <si>
+    <t>pathogen</t>
+  </si>
+  <si>
+    <t>codigo</t>
+  </si>
+  <si>
+    <t>Positivo</t>
+  </si>
+  <si>
+    <t>positivo</t>
   </si>
   <si>
     <t>codigo_externo_do_paciente</t>
@@ -349,13 +364,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -365,6 +383,9 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -668,13 +689,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -695,10 +716,10 @@
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="2"/>
@@ -707,10 +728,10 @@
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="2"/>
@@ -719,10 +740,10 @@
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="2"/>
@@ -731,10 +752,10 @@
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="2"/>
@@ -743,10 +764,10 @@
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="2"/>
@@ -755,10 +776,10 @@
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="2"/>
@@ -767,10 +788,10 @@
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="2"/>
@@ -779,10 +800,10 @@
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="2"/>
@@ -791,10 +812,10 @@
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="2"/>
@@ -803,10 +824,10 @@
       <c r="A11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="2"/>
@@ -815,10 +836,10 @@
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="2"/>
@@ -827,10 +848,10 @@
       <c r="A13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="2"/>
@@ -839,709 +860,709 @@
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>24</v>
       </c>
+      <c r="D14" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>24</v>
       </c>
+      <c r="D15" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="C16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>21</v>
+      <c r="B17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>6</v>
+      <c r="B18" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>9</v>
+      <c r="B19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>12</v>
+      <c r="B20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>32</v>
+      <c r="B22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="B23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="20.25">
-      <c r="A24" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D24" s="2"/>
+      <c r="D24" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="20.25">
+      <c r="A27" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>12</v>
+      <c r="C27" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="D27" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>21</v>
+        <v>42</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D28" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D29" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
-      <c r="A30" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
-      <c r="A31" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D31" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
-      <c r="A32" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="D32" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
       <c r="A33" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C33" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>48</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D33" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25">
       <c r="A34" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>34</v>
+      <c r="C34" s="3" t="s">
+        <v>50</v>
       </c>
       <c r="D34" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25">
       <c r="A35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="D35" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25">
       <c r="A36" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D36" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="17.25">
       <c r="A37" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B37" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>55</v>
+      <c r="C37" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="D37" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="17.25">
       <c r="A38" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="D38" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="17.25">
       <c r="A39" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B39" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="D39" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="17.25">
       <c r="A40" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="D40" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="17.25">
       <c r="A41" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="D41" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="17.25">
       <c r="A42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D42" s="2"/>
+      <c r="D42" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="17.25">
       <c r="A43" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>63</v>
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D43" s="2"/>
+        <v>39</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="17.25">
       <c r="A44" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>53</v>
+        <v>42</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="D44" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="17.25">
       <c r="A45" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="D45" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="17.25">
       <c r="A46" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="D46" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="17.25">
       <c r="A47" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D47" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="17.25">
       <c r="A48" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D48" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="17.25">
       <c r="A49" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D49" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="17.25">
       <c r="A50" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>12</v>
+        <v>42</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="17.25">
       <c r="A51" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>21</v>
+        <v>42</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="17.25">
       <c r="A52" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>15</v>
+        <v>42</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="17.25">
       <c r="A53" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>6</v>
+        <v>42</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="17.25">
       <c r="A54" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C54" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D54" s="2"/>
+      <c r="D54" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="17.25">
       <c r="A55" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D55" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="17.25">
       <c r="A56" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D56" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="17.25">
       <c r="A57" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>12</v>
+        <v>73</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D57" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="17.25">
       <c r="A58" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B58" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>6</v>
+      <c r="B58" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D58" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="17.25">
       <c r="A59" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>18</v>
+        <v>73</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D59" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="17.25">
       <c r="A60" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="D60" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="17.25">
       <c r="A61" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B61" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>18</v>
+      <c r="C61" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D61" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="17.25">
       <c r="A62" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B62" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B62" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D62" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="17.25">
       <c r="A63" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>15</v>
+        <v>73</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>81</v>
       </c>
       <c r="D63" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="17.25">
       <c r="A64" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>21</v>
+        <v>82</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D64" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="17.25">
       <c r="A65" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>6</v>
+        <v>82</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D65" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="17.25">
       <c r="A66" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>6</v>
+        <v>82</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D66" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="17.25">
       <c r="A67" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>12</v>
+        <v>82</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D67" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="17.25">
       <c r="A68" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>9</v>
+        <v>82</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D68" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="17.25">
       <c r="A69" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>30</v>
+        <v>82</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D69" s="2"/>
     </row>
@@ -1549,11 +1570,11 @@
       <c r="A70" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>40</v>
+      <c r="B70" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="D70" s="2"/>
     </row>
@@ -1561,11 +1582,11 @@
       <c r="A71" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B71" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>12</v>
+      <c r="B71" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D71" s="2"/>
     </row>
@@ -1573,169 +1594,205 @@
       <c r="A72" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B72" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>18</v>
+      <c r="B72" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="D72" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="17.25">
       <c r="A73" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>6</v>
+        <v>87</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="D73" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="17.25">
       <c r="A74" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>21</v>
+        <v>87</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="D74" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="17.25">
       <c r="A75" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>15</v>
+        <v>87</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D75" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="17.25">
       <c r="A76" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>9</v>
+        <v>87</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D76" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="17.25">
       <c r="A77" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>30</v>
+        <v>46</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="D77" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="17.25">
       <c r="A78" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>9</v>
+        <v>87</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D78" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="17.25">
       <c r="A79" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>15</v>
+        <v>87</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D79" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="17.25">
       <c r="A80" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>40</v>
+        <v>87</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="D80" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="17.25">
       <c r="A81" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>6</v>
+        <v>91</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D81" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="17.25">
       <c r="A82" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>12</v>
+        <v>91</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D82" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="17.25">
       <c r="A83" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>18</v>
+        <v>91</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="D83" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="17.25">
       <c r="A84" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B84" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D84" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="17.25">
+      <c r="A85" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D85" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="17.25">
+      <c r="A86" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D86" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="17.25">
+      <c r="A87" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B87" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C87" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D84" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
-      <c r="A85" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D85" s="2"/>
+      <c r="D87" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+      <c r="A88" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D88" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>